<commit_message>
Update staff list and KPI master templates using live Firestore data
</commit_message>
<xml_diff>
--- a/templates/template_Jamui.xlsx
+++ b/templates/template_Jamui.xlsx
@@ -1065,12 +1065,12 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Rakesh Singh</t>
+          <t>Rinki Kumari</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Senior Field Officer</t>
+          <t>Field Officer</t>
         </is>
       </c>
       <c r="D3" s="2">
@@ -1257,12 +1257,12 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Rakesh Singh</t>
+          <t>Rinki Kumari</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Senior Field Officer</t>
+          <t>Field Officer</t>
         </is>
       </c>
     </row>
@@ -1426,12 +1426,12 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Rakesh Singh</t>
+          <t>Rinki Kumari</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Senior Field Officer</t>
+          <t>Field Officer</t>
         </is>
       </c>
     </row>
@@ -1595,12 +1595,12 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Rakesh Singh</t>
+          <t>Rinki Kumari</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Senior Field Officer</t>
+          <t>Field Officer</t>
         </is>
       </c>
     </row>
@@ -1764,12 +1764,12 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Rakesh Singh</t>
+          <t>Rinki Kumari</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Senior Field Officer</t>
+          <t>Field Officer</t>
         </is>
       </c>
     </row>
@@ -1933,12 +1933,12 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Rakesh Singh</t>
+          <t>Rinki Kumari</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Senior Field Officer</t>
+          <t>Field Officer</t>
         </is>
       </c>
     </row>
@@ -2102,12 +2102,12 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Rakesh Singh</t>
+          <t>Rinki Kumari</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Senior Field Officer</t>
+          <t>Field Officer</t>
         </is>
       </c>
     </row>
@@ -2271,12 +2271,12 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Rakesh Singh</t>
+          <t>Rinki Kumari</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Senior Field Officer</t>
+          <t>Field Officer</t>
         </is>
       </c>
     </row>
@@ -2440,12 +2440,12 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Rakesh Singh</t>
+          <t>Rinki Kumari</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Senior Field Officer</t>
+          <t>Field Officer</t>
         </is>
       </c>
     </row>
@@ -2609,12 +2609,12 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Rakesh Singh</t>
+          <t>Rinki Kumari</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Senior Field Officer</t>
+          <t>Field Officer</t>
         </is>
       </c>
     </row>
@@ -2778,12 +2778,12 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Rakesh Singh</t>
+          <t>Rinki Kumari</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Senior Field Officer</t>
+          <t>Field Officer</t>
         </is>
       </c>
     </row>
@@ -2946,7 +2946,7 @@
       </c>
       <c r="AB1" s="3" t="inlineStr">
         <is>
-          <t>Rakesh Singh</t>
+          <t>Rinki Kumari</t>
         </is>
       </c>
     </row>
@@ -3081,12 +3081,12 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Rakesh Singh</t>
+          <t>Rinki Kumari</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Senior Field Officer</t>
+          <t>Field Officer</t>
         </is>
       </c>
       <c r="C3" s="2">
@@ -3576,12 +3576,12 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Rakesh Singh</t>
+          <t>Rinki Kumari</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Senior Field Officer</t>
+          <t>Field Officer</t>
         </is>
       </c>
     </row>
@@ -3745,12 +3745,12 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Rakesh Singh</t>
+          <t>Rinki Kumari</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Senior Field Officer</t>
+          <t>Field Officer</t>
         </is>
       </c>
     </row>
@@ -3914,12 +3914,12 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Rakesh Singh</t>
+          <t>Rinki Kumari</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Senior Field Officer</t>
+          <t>Field Officer</t>
         </is>
       </c>
     </row>
@@ -4083,12 +4083,12 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Rakesh Singh</t>
+          <t>Rinki Kumari</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Senior Field Officer</t>
+          <t>Field Officer</t>
         </is>
       </c>
     </row>
@@ -4252,12 +4252,12 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Rakesh Singh</t>
+          <t>Rinki Kumari</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Senior Field Officer</t>
+          <t>Field Officer</t>
         </is>
       </c>
     </row>
@@ -4421,12 +4421,12 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Rakesh Singh</t>
+          <t>Rinki Kumari</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Senior Field Officer</t>
+          <t>Field Officer</t>
         </is>
       </c>
     </row>
@@ -4590,12 +4590,12 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Rakesh Singh</t>
+          <t>Rinki Kumari</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Senior Field Officer</t>
+          <t>Field Officer</t>
         </is>
       </c>
     </row>
@@ -4759,12 +4759,12 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Rakesh Singh</t>
+          <t>Rinki Kumari</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Senior Field Officer</t>
+          <t>Field Officer</t>
         </is>
       </c>
     </row>
@@ -4928,12 +4928,12 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Rakesh Singh</t>
+          <t>Rinki Kumari</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Senior Field Officer</t>
+          <t>Field Officer</t>
         </is>
       </c>
     </row>
@@ -5097,12 +5097,12 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Rakesh Singh</t>
+          <t>Rinki Kumari</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Senior Field Officer</t>
+          <t>Field Officer</t>
         </is>
       </c>
     </row>
@@ -5266,12 +5266,12 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Rakesh Singh</t>
+          <t>Rinki Kumari</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Senior Field Officer</t>
+          <t>Field Officer</t>
         </is>
       </c>
     </row>
@@ -5435,12 +5435,12 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Rakesh Singh</t>
+          <t>Rinki Kumari</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Senior Field Officer</t>
+          <t>Field Officer</t>
         </is>
       </c>
     </row>
@@ -5604,12 +5604,12 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Rakesh Singh</t>
+          <t>Rinki Kumari</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Senior Field Officer</t>
+          <t>Field Officer</t>
         </is>
       </c>
     </row>
@@ -5773,12 +5773,12 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Rakesh Singh</t>
+          <t>Rinki Kumari</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Senior Field Officer</t>
+          <t>Field Officer</t>
         </is>
       </c>
     </row>
@@ -5942,12 +5942,12 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Rakesh Singh</t>
+          <t>Rinki Kumari</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Senior Field Officer</t>
+          <t>Field Officer</t>
         </is>
       </c>
     </row>
@@ -6111,12 +6111,12 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Rakesh Singh</t>
+          <t>Rinki Kumari</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Senior Field Officer</t>
+          <t>Field Officer</t>
         </is>
       </c>
     </row>
@@ -6280,12 +6280,12 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Rakesh Singh</t>
+          <t>Rinki Kumari</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Senior Field Officer</t>
+          <t>Field Officer</t>
         </is>
       </c>
     </row>
@@ -6449,12 +6449,12 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Rakesh Singh</t>
+          <t>Rinki Kumari</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Senior Field Officer</t>
+          <t>Field Officer</t>
         </is>
       </c>
     </row>
@@ -6618,12 +6618,12 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Rakesh Singh</t>
+          <t>Rinki Kumari</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Senior Field Officer</t>
+          <t>Field Officer</t>
         </is>
       </c>
     </row>
@@ -6787,12 +6787,12 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Rakesh Singh</t>
+          <t>Rinki Kumari</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Senior Field Officer</t>
+          <t>Field Officer</t>
         </is>
       </c>
     </row>
@@ -6956,12 +6956,12 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Rakesh Singh</t>
+          <t>Rinki Kumari</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Senior Field Officer</t>
+          <t>Field Officer</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Centralize staff directory in Firebase and update templates for new districts
</commit_message>
<xml_diff>
--- a/templates/template_Jamui.xlsx
+++ b/templates/template_Jamui.xlsx
@@ -965,7 +965,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I3"/>
+  <dimension ref="A1:I5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -1029,12 +1029,12 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Rajiv Kumar</t>
+          <t>Bablu Kumar</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Field Officer</t>
+          <t>FC</t>
         </is>
       </c>
       <c r="D2" s="2">
@@ -1065,12 +1065,12 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Rinki Kumari</t>
+          <t>Monu Kumar</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Field Officer</t>
+          <t>FC</t>
         </is>
       </c>
       <c r="D3" s="2">
@@ -1095,6 +1095,78 @@
       </c>
       <c r="I3" s="2">
         <f>'CONSOLIDATED SHEET'!H3</f>
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Rajiv Kumar</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>FC</t>
+        </is>
+      </c>
+      <c r="D4" s="2">
+        <f>'CONSOLIDATED SHEET'!C4</f>
+        <v/>
+      </c>
+      <c r="E4" s="2">
+        <f>'CONSOLIDATED SHEET'!D4</f>
+        <v/>
+      </c>
+      <c r="F4" s="2">
+        <f>'CONSOLIDATED SHEET'!E4</f>
+        <v/>
+      </c>
+      <c r="G4" s="2">
+        <f>'CONSOLIDATED SHEET'!F4</f>
+        <v/>
+      </c>
+      <c r="H4" s="2">
+        <f>'CONSOLIDATED SHEET'!G4</f>
+        <v/>
+      </c>
+      <c r="I4" s="2">
+        <f>'CONSOLIDATED SHEET'!H4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Rinki Kumari</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>FC</t>
+        </is>
+      </c>
+      <c r="D5" s="2">
+        <f>'CONSOLIDATED SHEET'!C5</f>
+        <v/>
+      </c>
+      <c r="E5" s="2">
+        <f>'CONSOLIDATED SHEET'!D5</f>
+        <v/>
+      </c>
+      <c r="F5" s="2">
+        <f>'CONSOLIDATED SHEET'!E5</f>
+        <v/>
+      </c>
+      <c r="G5" s="2">
+        <f>'CONSOLIDATED SHEET'!F5</f>
+        <v/>
+      </c>
+      <c r="H5" s="2">
+        <f>'CONSOLIDATED SHEET'!G5</f>
+        <v/>
+      </c>
+      <c r="I5" s="2">
+        <f>'CONSOLIDATED SHEET'!H5</f>
         <v/>
       </c>
     </row>
@@ -1109,7 +1181,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U42"/>
+  <dimension ref="A1:U122"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -1245,24 +1317,48 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Rajiv Kumar</t>
+          <t>Bablu Kumar</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Field Officer</t>
+          <t>FC</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
+          <t>Monu Kumar</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>FC</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="inlineStr">
+        <is>
+          <t>Rajiv Kumar</t>
+        </is>
+      </c>
+      <c r="B82" s="2" t="inlineStr">
+        <is>
+          <t>FC</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="2" t="inlineStr">
+        <is>
           <t>Rinki Kumari</t>
         </is>
       </c>
-      <c r="B42" s="2" t="inlineStr">
-        <is>
-          <t>Field Officer</t>
+      <c r="B122" s="2" t="inlineStr">
+        <is>
+          <t>FC</t>
         </is>
       </c>
     </row>
@@ -1278,7 +1374,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U42"/>
+  <dimension ref="A1:U122"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -1414,24 +1510,48 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Rajiv Kumar</t>
+          <t>Bablu Kumar</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Field Officer</t>
+          <t>FC</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
+          <t>Monu Kumar</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>FC</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="inlineStr">
+        <is>
+          <t>Rajiv Kumar</t>
+        </is>
+      </c>
+      <c r="B82" s="2" t="inlineStr">
+        <is>
+          <t>FC</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="2" t="inlineStr">
+        <is>
           <t>Rinki Kumari</t>
         </is>
       </c>
-      <c r="B42" s="2" t="inlineStr">
-        <is>
-          <t>Field Officer</t>
+      <c r="B122" s="2" t="inlineStr">
+        <is>
+          <t>FC</t>
         </is>
       </c>
     </row>
@@ -1447,7 +1567,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U42"/>
+  <dimension ref="A1:U122"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -1583,24 +1703,48 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Rajiv Kumar</t>
+          <t>Bablu Kumar</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Field Officer</t>
+          <t>FC</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
+          <t>Monu Kumar</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>FC</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="inlineStr">
+        <is>
+          <t>Rajiv Kumar</t>
+        </is>
+      </c>
+      <c r="B82" s="2" t="inlineStr">
+        <is>
+          <t>FC</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="2" t="inlineStr">
+        <is>
           <t>Rinki Kumari</t>
         </is>
       </c>
-      <c r="B42" s="2" t="inlineStr">
-        <is>
-          <t>Field Officer</t>
+      <c r="B122" s="2" t="inlineStr">
+        <is>
+          <t>FC</t>
         </is>
       </c>
     </row>
@@ -1616,7 +1760,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U42"/>
+  <dimension ref="A1:U122"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -1752,24 +1896,48 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Rajiv Kumar</t>
+          <t>Bablu Kumar</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Field Officer</t>
+          <t>FC</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
+          <t>Monu Kumar</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>FC</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="inlineStr">
+        <is>
+          <t>Rajiv Kumar</t>
+        </is>
+      </c>
+      <c r="B82" s="2" t="inlineStr">
+        <is>
+          <t>FC</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="2" t="inlineStr">
+        <is>
           <t>Rinki Kumari</t>
         </is>
       </c>
-      <c r="B42" s="2" t="inlineStr">
-        <is>
-          <t>Field Officer</t>
+      <c r="B122" s="2" t="inlineStr">
+        <is>
+          <t>FC</t>
         </is>
       </c>
     </row>
@@ -1785,7 +1953,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U42"/>
+  <dimension ref="A1:U122"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -1921,24 +2089,48 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Rajiv Kumar</t>
+          <t>Bablu Kumar</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Field Officer</t>
+          <t>FC</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
+          <t>Monu Kumar</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>FC</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="inlineStr">
+        <is>
+          <t>Rajiv Kumar</t>
+        </is>
+      </c>
+      <c r="B82" s="2" t="inlineStr">
+        <is>
+          <t>FC</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="2" t="inlineStr">
+        <is>
           <t>Rinki Kumari</t>
         </is>
       </c>
-      <c r="B42" s="2" t="inlineStr">
-        <is>
-          <t>Field Officer</t>
+      <c r="B122" s="2" t="inlineStr">
+        <is>
+          <t>FC</t>
         </is>
       </c>
     </row>
@@ -1954,7 +2146,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U42"/>
+  <dimension ref="A1:U122"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -2090,24 +2282,48 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Rajiv Kumar</t>
+          <t>Bablu Kumar</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Field Officer</t>
+          <t>FC</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
+          <t>Monu Kumar</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>FC</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="inlineStr">
+        <is>
+          <t>Rajiv Kumar</t>
+        </is>
+      </c>
+      <c r="B82" s="2" t="inlineStr">
+        <is>
+          <t>FC</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="2" t="inlineStr">
+        <is>
           <t>Rinki Kumari</t>
         </is>
       </c>
-      <c r="B42" s="2" t="inlineStr">
-        <is>
-          <t>Field Officer</t>
+      <c r="B122" s="2" t="inlineStr">
+        <is>
+          <t>FC</t>
         </is>
       </c>
     </row>
@@ -2123,7 +2339,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U42"/>
+  <dimension ref="A1:U122"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -2259,24 +2475,48 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Rajiv Kumar</t>
+          <t>Bablu Kumar</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Field Officer</t>
+          <t>FC</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
+          <t>Monu Kumar</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>FC</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="inlineStr">
+        <is>
+          <t>Rajiv Kumar</t>
+        </is>
+      </c>
+      <c r="B82" s="2" t="inlineStr">
+        <is>
+          <t>FC</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="2" t="inlineStr">
+        <is>
           <t>Rinki Kumari</t>
         </is>
       </c>
-      <c r="B42" s="2" t="inlineStr">
-        <is>
-          <t>Field Officer</t>
+      <c r="B122" s="2" t="inlineStr">
+        <is>
+          <t>FC</t>
         </is>
       </c>
     </row>
@@ -2292,7 +2532,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U42"/>
+  <dimension ref="A1:U122"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -2428,24 +2668,48 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Rajiv Kumar</t>
+          <t>Bablu Kumar</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Field Officer</t>
+          <t>FC</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
+          <t>Monu Kumar</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>FC</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="inlineStr">
+        <is>
+          <t>Rajiv Kumar</t>
+        </is>
+      </c>
+      <c r="B82" s="2" t="inlineStr">
+        <is>
+          <t>FC</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="2" t="inlineStr">
+        <is>
           <t>Rinki Kumari</t>
         </is>
       </c>
-      <c r="B42" s="2" t="inlineStr">
-        <is>
-          <t>Field Officer</t>
+      <c r="B122" s="2" t="inlineStr">
+        <is>
+          <t>FC</t>
         </is>
       </c>
     </row>
@@ -2461,7 +2725,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U42"/>
+  <dimension ref="A1:U122"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -2597,24 +2861,48 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Rajiv Kumar</t>
+          <t>Bablu Kumar</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Field Officer</t>
+          <t>FC</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
+          <t>Monu Kumar</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>FC</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="inlineStr">
+        <is>
+          <t>Rajiv Kumar</t>
+        </is>
+      </c>
+      <c r="B82" s="2" t="inlineStr">
+        <is>
+          <t>FC</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="2" t="inlineStr">
+        <is>
           <t>Rinki Kumari</t>
         </is>
       </c>
-      <c r="B42" s="2" t="inlineStr">
-        <is>
-          <t>Field Officer</t>
+      <c r="B122" s="2" t="inlineStr">
+        <is>
+          <t>FC</t>
         </is>
       </c>
     </row>
@@ -2630,7 +2918,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U42"/>
+  <dimension ref="A1:U122"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -2766,24 +3054,48 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Rajiv Kumar</t>
+          <t>Bablu Kumar</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Field Officer</t>
+          <t>FC</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
+          <t>Monu Kumar</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>FC</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="inlineStr">
+        <is>
+          <t>Rajiv Kumar</t>
+        </is>
+      </c>
+      <c r="B82" s="2" t="inlineStr">
+        <is>
+          <t>FC</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="2" t="inlineStr">
+        <is>
           <t>Rinki Kumari</t>
         </is>
       </c>
-      <c r="B42" s="2" t="inlineStr">
-        <is>
-          <t>Field Officer</t>
+      <c r="B122" s="2" t="inlineStr">
+        <is>
+          <t>FC</t>
         </is>
       </c>
     </row>
@@ -2799,7 +3111,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE33"/>
+  <dimension ref="A1:AO33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -2831,6 +3143,14 @@
     <col width="13" customWidth="1" min="29" max="29"/>
     <col width="13" customWidth="1" min="30" max="30"/>
     <col width="13" customWidth="1" min="31" max="31"/>
+    <col width="13" customWidth="1" min="33" max="33"/>
+    <col width="13" customWidth="1" min="34" max="34"/>
+    <col width="13" customWidth="1" min="35" max="35"/>
+    <col width="13" customWidth="1" min="36" max="36"/>
+    <col width="13" customWidth="1" min="38" max="38"/>
+    <col width="13" customWidth="1" min="39" max="39"/>
+    <col width="13" customWidth="1" min="40" max="40"/>
+    <col width="13" customWidth="1" min="41" max="41"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2941,10 +3261,20 @@
       </c>
       <c r="W1" s="3" t="inlineStr">
         <is>
+          <t>Bablu Kumar</t>
+        </is>
+      </c>
+      <c r="AB1" s="3" t="inlineStr">
+        <is>
+          <t>Monu Kumar</t>
+        </is>
+      </c>
+      <c r="AG1" s="3" t="inlineStr">
+        <is>
           <t>Rajiv Kumar</t>
         </is>
       </c>
-      <c r="AB1" s="3" t="inlineStr">
+      <c r="AL1" s="3" t="inlineStr">
         <is>
           <t>Rinki Kumari</t>
         </is>
@@ -2953,12 +3283,12 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Rajiv Kumar</t>
+          <t>Bablu Kumar</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Field Officer</t>
+          <t>FC</t>
         </is>
       </c>
       <c r="C2" s="2">
@@ -3077,16 +3407,56 @@
           <t>DBT</t>
         </is>
       </c>
+      <c r="AG2" s="3" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="AH2" s="3" t="inlineStr">
+        <is>
+          <t>Reported By</t>
+        </is>
+      </c>
+      <c r="AI2" s="3" t="inlineStr">
+        <is>
+          <t>HIV</t>
+        </is>
+      </c>
+      <c r="AJ2" s="3" t="inlineStr">
+        <is>
+          <t>DBT</t>
+        </is>
+      </c>
+      <c r="AL2" s="3" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="AM2" s="3" t="inlineStr">
+        <is>
+          <t>Reported By</t>
+        </is>
+      </c>
+      <c r="AN2" s="3" t="inlineStr">
+        <is>
+          <t>HIV</t>
+        </is>
+      </c>
+      <c r="AO2" s="3" t="inlineStr">
+        <is>
+          <t>DBT</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Rinki Kumari</t>
+          <t>Monu Kumar</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Field Officer</t>
+          <t>FC</t>
         </is>
       </c>
       <c r="C3" s="2">
@@ -3171,20 +3541,210 @@
       <c r="AB3" s="4" t="n">
         <v>1</v>
       </c>
+      <c r="AG3" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AL3" s="4" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Rajiv Kumar</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>FC</t>
+        </is>
+      </c>
+      <c r="C4" s="2">
+        <f>COUNTA('1ST'!C82:C121)+COUNTA('2nd'!C82:C121)+COUNTA('3rd'!C82:C121)+COUNTA('4th'!C82:C121)+COUNTA('5th'!C82:C121)+COUNTA('6th'!C82:C121)+COUNTA('7th'!C82:C121)+COUNTA('8th'!C82:C121)+COUNTA('9th'!C82:C121)+COUNTA('10th'!C82:C121)+COUNTA('11th'!C82:C121)+COUNTA('12th'!C82:C121)+COUNTA('13th'!C82:C121)+COUNTA('14th'!C82:C121)+COUNTA('15th'!C82:C121)+COUNTA('16th'!C82:C121)+COUNTA('17th'!C82:C121)+COUNTA('18th'!C82:C121)+COUNTA('19th'!C82:C121)+COUNTA('20th'!C82:C121)+COUNTA('21st'!C82:C121)+COUNTA('22nd'!C82:C121)+COUNTA('23rd'!C82:C121)+COUNTA('24th'!C82:C121)+COUNTA('25th'!C82:C121)+COUNTA('26th'!C82:C121)+COUNTA('27th'!C82:C121)+COUNTA('28th'!C82:C121)+COUNTA('29th'!C82:C121)+COUNTA('30th'!C82:C121)+COUNTA('31st'!C82:C121)</f>
+        <v/>
+      </c>
+      <c r="D4" s="2">
+        <f>COUNTA('1ST'!D82:D121)+COUNTA('2nd'!D82:D121)+COUNTA('3rd'!D82:D121)+COUNTA('4th'!D82:D121)+COUNTA('5th'!D82:D121)+COUNTA('6th'!D82:D121)+COUNTA('7th'!D82:D121)+COUNTA('8th'!D82:D121)+COUNTA('9th'!D82:D121)+COUNTA('10th'!D82:D121)+COUNTA('11th'!D82:D121)+COUNTA('12th'!D82:D121)+COUNTA('13th'!D82:D121)+COUNTA('14th'!D82:D121)+COUNTA('15th'!D82:D121)+COUNTA('16th'!D82:D121)+COUNTA('17th'!D82:D121)+COUNTA('18th'!D82:D121)+COUNTA('19th'!D82:D121)+COUNTA('20th'!D82:D121)+COUNTA('21st'!D82:D121)+COUNTA('22nd'!D82:D121)+COUNTA('23rd'!D82:D121)+COUNTA('24th'!D82:D121)+COUNTA('25th'!D82:D121)+COUNTA('26th'!D82:D121)+COUNTA('27th'!D82:D121)+COUNTA('28th'!D82:D121)+COUNTA('29th'!D82:D121)+COUNTA('30th'!D82:D121)+COUNTA('31st'!D82:D121)</f>
+        <v/>
+      </c>
+      <c r="E4" s="2">
+        <f>COUNTA('1ST'!E82:E121)+COUNTA('2nd'!E82:E121)+COUNTA('3rd'!E82:E121)+COUNTA('4th'!E82:E121)+COUNTA('5th'!E82:E121)+COUNTA('6th'!E82:E121)+COUNTA('7th'!E82:E121)+COUNTA('8th'!E82:E121)+COUNTA('9th'!E82:E121)+COUNTA('10th'!E82:E121)+COUNTA('11th'!E82:E121)+COUNTA('12th'!E82:E121)+COUNTA('13th'!E82:E121)+COUNTA('14th'!E82:E121)+COUNTA('15th'!E82:E121)+COUNTA('16th'!E82:E121)+COUNTA('17th'!E82:E121)+COUNTA('18th'!E82:E121)+COUNTA('19th'!E82:E121)+COUNTA('20th'!E82:E121)+COUNTA('21st'!E82:E121)+COUNTA('22nd'!E82:E121)+COUNTA('23rd'!E82:E121)+COUNTA('24th'!E82:E121)+COUNTA('25th'!E82:E121)+COUNTA('26th'!E82:E121)+COUNTA('27th'!E82:E121)+COUNTA('28th'!E82:E121)+COUNTA('29th'!E82:E121)+COUNTA('30th'!E82:E121)+COUNTA('31st'!E82:E121)</f>
+        <v/>
+      </c>
+      <c r="F4" s="2">
+        <f>COUNTA('1ST'!F82:F121)+COUNTA('2nd'!F82:F121)+COUNTA('3rd'!F82:F121)+COUNTA('4th'!F82:F121)+COUNTA('5th'!F82:F121)+COUNTA('6th'!F82:F121)+COUNTA('7th'!F82:F121)+COUNTA('8th'!F82:F121)+COUNTA('9th'!F82:F121)+COUNTA('10th'!F82:F121)+COUNTA('11th'!F82:F121)+COUNTA('12th'!F82:F121)+COUNTA('13th'!F82:F121)+COUNTA('14th'!F82:F121)+COUNTA('15th'!F82:F121)+COUNTA('16th'!F82:F121)+COUNTA('17th'!F82:F121)+COUNTA('18th'!F82:F121)+COUNTA('19th'!F82:F121)+COUNTA('20th'!F82:F121)+COUNTA('21st'!F82:F121)+COUNTA('22nd'!F82:F121)+COUNTA('23rd'!F82:F121)+COUNTA('24th'!F82:F121)+COUNTA('25th'!F82:F121)+COUNTA('26th'!F82:F121)+COUNTA('27th'!F82:F121)+COUNTA('28th'!F82:F121)+COUNTA('29th'!F82:F121)+COUNTA('30th'!F82:F121)+COUNTA('31st'!F82:F121)</f>
+        <v/>
+      </c>
+      <c r="G4" s="2">
+        <f>COUNTA('1ST'!G82:G121)+COUNTA('2nd'!G82:G121)+COUNTA('3rd'!G82:G121)+COUNTA('4th'!G82:G121)+COUNTA('5th'!G82:G121)+COUNTA('6th'!G82:G121)+COUNTA('7th'!G82:G121)+COUNTA('8th'!G82:G121)+COUNTA('9th'!G82:G121)+COUNTA('10th'!G82:G121)+COUNTA('11th'!G82:G121)+COUNTA('12th'!G82:G121)+COUNTA('13th'!G82:G121)+COUNTA('14th'!G82:G121)+COUNTA('15th'!G82:G121)+COUNTA('16th'!G82:G121)+COUNTA('17th'!G82:G121)+COUNTA('18th'!G82:G121)+COUNTA('19th'!G82:G121)+COUNTA('20th'!G82:G121)+COUNTA('21st'!G82:G121)+COUNTA('22nd'!G82:G121)+COUNTA('23rd'!G82:G121)+COUNTA('24th'!G82:G121)+COUNTA('25th'!G82:G121)+COUNTA('26th'!G82:G121)+COUNTA('27th'!G82:G121)+COUNTA('28th'!G82:G121)+COUNTA('29th'!G82:G121)+COUNTA('30th'!G82:G121)+COUNTA('31st'!G82:G121)</f>
+        <v/>
+      </c>
+      <c r="H4" s="2">
+        <f>COUNTA('1ST'!H82:H121)+COUNTA('2nd'!H82:H121)+COUNTA('3rd'!H82:H121)+COUNTA('4th'!H82:H121)+COUNTA('5th'!H82:H121)+COUNTA('6th'!H82:H121)+COUNTA('7th'!H82:H121)+COUNTA('8th'!H82:H121)+COUNTA('9th'!H82:H121)+COUNTA('10th'!H82:H121)+COUNTA('11th'!H82:H121)+COUNTA('12th'!H82:H121)+COUNTA('13th'!H82:H121)+COUNTA('14th'!H82:H121)+COUNTA('15th'!H82:H121)+COUNTA('16th'!H82:H121)+COUNTA('17th'!H82:H121)+COUNTA('18th'!H82:H121)+COUNTA('19th'!H82:H121)+COUNTA('20th'!H82:H121)+COUNTA('21st'!H82:H121)+COUNTA('22nd'!H82:H121)+COUNTA('23rd'!H82:H121)+COUNTA('24th'!H82:H121)+COUNTA('25th'!H82:H121)+COUNTA('26th'!H82:H121)+COUNTA('27th'!H82:H121)+COUNTA('28th'!H82:H121)+COUNTA('29th'!H82:H121)+COUNTA('30th'!H82:H121)+COUNTA('31st'!H82:H121)</f>
+        <v/>
+      </c>
+      <c r="I4" s="2">
+        <f>COUNTA('1ST'!I82:I121)+COUNTA('2nd'!I82:I121)+COUNTA('3rd'!I82:I121)+COUNTA('4th'!I82:I121)+COUNTA('5th'!I82:I121)+COUNTA('6th'!I82:I121)+COUNTA('7th'!I82:I121)+COUNTA('8th'!I82:I121)+COUNTA('9th'!I82:I121)+COUNTA('10th'!I82:I121)+COUNTA('11th'!I82:I121)+COUNTA('12th'!I82:I121)+COUNTA('13th'!I82:I121)+COUNTA('14th'!I82:I121)+COUNTA('15th'!I82:I121)+COUNTA('16th'!I82:I121)+COUNTA('17th'!I82:I121)+COUNTA('18th'!I82:I121)+COUNTA('19th'!I82:I121)+COUNTA('20th'!I82:I121)+COUNTA('21st'!I82:I121)+COUNTA('22nd'!I82:I121)+COUNTA('23rd'!I82:I121)+COUNTA('24th'!I82:I121)+COUNTA('25th'!I82:I121)+COUNTA('26th'!I82:I121)+COUNTA('27th'!I82:I121)+COUNTA('28th'!I82:I121)+COUNTA('29th'!I82:I121)+COUNTA('30th'!I82:I121)+COUNTA('31st'!I82:I121)</f>
+        <v/>
+      </c>
+      <c r="J4" s="2">
+        <f>COUNTA('1ST'!J82:J121)+COUNTA('2nd'!J82:J121)+COUNTA('3rd'!J82:J121)+COUNTA('4th'!J82:J121)+COUNTA('5th'!J82:J121)+COUNTA('6th'!J82:J121)+COUNTA('7th'!J82:J121)+COUNTA('8th'!J82:J121)+COUNTA('9th'!J82:J121)+COUNTA('10th'!J82:J121)+COUNTA('11th'!J82:J121)+COUNTA('12th'!J82:J121)+COUNTA('13th'!J82:J121)+COUNTA('14th'!J82:J121)+COUNTA('15th'!J82:J121)+COUNTA('16th'!J82:J121)+COUNTA('17th'!J82:J121)+COUNTA('18th'!J82:J121)+COUNTA('19th'!J82:J121)+COUNTA('20th'!J82:J121)+COUNTA('21st'!J82:J121)+COUNTA('22nd'!J82:J121)+COUNTA('23rd'!J82:J121)+COUNTA('24th'!J82:J121)+COUNTA('25th'!J82:J121)+COUNTA('26th'!J82:J121)+COUNTA('27th'!J82:J121)+COUNTA('28th'!J82:J121)+COUNTA('29th'!J82:J121)+COUNTA('30th'!J82:J121)+COUNTA('31st'!J82:J121)</f>
+        <v/>
+      </c>
+      <c r="K4" s="2">
+        <f>COUNTA('1ST'!K82:K121)+COUNTA('2nd'!K82:K121)+COUNTA('3rd'!K82:K121)+COUNTA('4th'!K82:K121)+COUNTA('5th'!K82:K121)+COUNTA('6th'!K82:K121)+COUNTA('7th'!K82:K121)+COUNTA('8th'!K82:K121)+COUNTA('9th'!K82:K121)+COUNTA('10th'!K82:K121)+COUNTA('11th'!K82:K121)+COUNTA('12th'!K82:K121)+COUNTA('13th'!K82:K121)+COUNTA('14th'!K82:K121)+COUNTA('15th'!K82:K121)+COUNTA('16th'!K82:K121)+COUNTA('17th'!K82:K121)+COUNTA('18th'!K82:K121)+COUNTA('19th'!K82:K121)+COUNTA('20th'!K82:K121)+COUNTA('21st'!K82:K121)+COUNTA('22nd'!K82:K121)+COUNTA('23rd'!K82:K121)+COUNTA('24th'!K82:K121)+COUNTA('25th'!K82:K121)+COUNTA('26th'!K82:K121)+COUNTA('27th'!K82:K121)+COUNTA('28th'!K82:K121)+COUNTA('29th'!K82:K121)+COUNTA('30th'!K82:K121)+COUNTA('31st'!K82:K121)</f>
+        <v/>
+      </c>
+      <c r="L4" s="2">
+        <f>COUNTA('1ST'!L82:L121)+COUNTA('2nd'!L82:L121)+COUNTA('3rd'!L82:L121)+COUNTA('4th'!L82:L121)+COUNTA('5th'!L82:L121)+COUNTA('6th'!L82:L121)+COUNTA('7th'!L82:L121)+COUNTA('8th'!L82:L121)+COUNTA('9th'!L82:L121)+COUNTA('10th'!L82:L121)+COUNTA('11th'!L82:L121)+COUNTA('12th'!L82:L121)+COUNTA('13th'!L82:L121)+COUNTA('14th'!L82:L121)+COUNTA('15th'!L82:L121)+COUNTA('16th'!L82:L121)+COUNTA('17th'!L82:L121)+COUNTA('18th'!L82:L121)+COUNTA('19th'!L82:L121)+COUNTA('20th'!L82:L121)+COUNTA('21st'!L82:L121)+COUNTA('22nd'!L82:L121)+COUNTA('23rd'!L82:L121)+COUNTA('24th'!L82:L121)+COUNTA('25th'!L82:L121)+COUNTA('26th'!L82:L121)+COUNTA('27th'!L82:L121)+COUNTA('28th'!L82:L121)+COUNTA('29th'!L82:L121)+COUNTA('30th'!L82:L121)+COUNTA('31st'!L82:L121)</f>
+        <v/>
+      </c>
+      <c r="M4" s="2">
+        <f>COUNTA('1ST'!M82:M121)+COUNTA('2nd'!M82:M121)+COUNTA('3rd'!M82:M121)+COUNTA('4th'!M82:M121)+COUNTA('5th'!M82:M121)+COUNTA('6th'!M82:M121)+COUNTA('7th'!M82:M121)+COUNTA('8th'!M82:M121)+COUNTA('9th'!M82:M121)+COUNTA('10th'!M82:M121)+COUNTA('11th'!M82:M121)+COUNTA('12th'!M82:M121)+COUNTA('13th'!M82:M121)+COUNTA('14th'!M82:M121)+COUNTA('15th'!M82:M121)+COUNTA('16th'!M82:M121)+COUNTA('17th'!M82:M121)+COUNTA('18th'!M82:M121)+COUNTA('19th'!M82:M121)+COUNTA('20th'!M82:M121)+COUNTA('21st'!M82:M121)+COUNTA('22nd'!M82:M121)+COUNTA('23rd'!M82:M121)+COUNTA('24th'!M82:M121)+COUNTA('25th'!M82:M121)+COUNTA('26th'!M82:M121)+COUNTA('27th'!M82:M121)+COUNTA('28th'!M82:M121)+COUNTA('29th'!M82:M121)+COUNTA('30th'!M82:M121)+COUNTA('31st'!M82:M121)</f>
+        <v/>
+      </c>
+      <c r="N4" s="2">
+        <f>COUNTA('1ST'!N82:N121)+COUNTA('2nd'!N82:N121)+COUNTA('3rd'!N82:N121)+COUNTA('4th'!N82:N121)+COUNTA('5th'!N82:N121)+COUNTA('6th'!N82:N121)+COUNTA('7th'!N82:N121)+COUNTA('8th'!N82:N121)+COUNTA('9th'!N82:N121)+COUNTA('10th'!N82:N121)+COUNTA('11th'!N82:N121)+COUNTA('12th'!N82:N121)+COUNTA('13th'!N82:N121)+COUNTA('14th'!N82:N121)+COUNTA('15th'!N82:N121)+COUNTA('16th'!N82:N121)+COUNTA('17th'!N82:N121)+COUNTA('18th'!N82:N121)+COUNTA('19th'!N82:N121)+COUNTA('20th'!N82:N121)+COUNTA('21st'!N82:N121)+COUNTA('22nd'!N82:N121)+COUNTA('23rd'!N82:N121)+COUNTA('24th'!N82:N121)+COUNTA('25th'!N82:N121)+COUNTA('26th'!N82:N121)+COUNTA('27th'!N82:N121)+COUNTA('28th'!N82:N121)+COUNTA('29th'!N82:N121)+COUNTA('30th'!N82:N121)+COUNTA('31st'!N82:N121)</f>
+        <v/>
+      </c>
+      <c r="O4" s="2">
+        <f>COUNTA('1ST'!O82:O121)+COUNTA('2nd'!O82:O121)+COUNTA('3rd'!O82:O121)+COUNTA('4th'!O82:O121)+COUNTA('5th'!O82:O121)+COUNTA('6th'!O82:O121)+COUNTA('7th'!O82:O121)+COUNTA('8th'!O82:O121)+COUNTA('9th'!O82:O121)+COUNTA('10th'!O82:O121)+COUNTA('11th'!O82:O121)+COUNTA('12th'!O82:O121)+COUNTA('13th'!O82:O121)+COUNTA('14th'!O82:O121)+COUNTA('15th'!O82:O121)+COUNTA('16th'!O82:O121)+COUNTA('17th'!O82:O121)+COUNTA('18th'!O82:O121)+COUNTA('19th'!O82:O121)+COUNTA('20th'!O82:O121)+COUNTA('21st'!O82:O121)+COUNTA('22nd'!O82:O121)+COUNTA('23rd'!O82:O121)+COUNTA('24th'!O82:O121)+COUNTA('25th'!O82:O121)+COUNTA('26th'!O82:O121)+COUNTA('27th'!O82:O121)+COUNTA('28th'!O82:O121)+COUNTA('29th'!O82:O121)+COUNTA('30th'!O82:O121)+COUNTA('31st'!O82:O121)</f>
+        <v/>
+      </c>
+      <c r="P4" s="2">
+        <f>COUNTA('1ST'!P82:P121)+COUNTA('2nd'!P82:P121)+COUNTA('3rd'!P82:P121)+COUNTA('4th'!P82:P121)+COUNTA('5th'!P82:P121)+COUNTA('6th'!P82:P121)+COUNTA('7th'!P82:P121)+COUNTA('8th'!P82:P121)+COUNTA('9th'!P82:P121)+COUNTA('10th'!P82:P121)+COUNTA('11th'!P82:P121)+COUNTA('12th'!P82:P121)+COUNTA('13th'!P82:P121)+COUNTA('14th'!P82:P121)+COUNTA('15th'!P82:P121)+COUNTA('16th'!P82:P121)+COUNTA('17th'!P82:P121)+COUNTA('18th'!P82:P121)+COUNTA('19th'!P82:P121)+COUNTA('20th'!P82:P121)+COUNTA('21st'!P82:P121)+COUNTA('22nd'!P82:P121)+COUNTA('23rd'!P82:P121)+COUNTA('24th'!P82:P121)+COUNTA('25th'!P82:P121)+COUNTA('26th'!P82:P121)+COUNTA('27th'!P82:P121)+COUNTA('28th'!P82:P121)+COUNTA('29th'!P82:P121)+COUNTA('30th'!P82:P121)+COUNTA('31st'!P82:P121)</f>
+        <v/>
+      </c>
+      <c r="Q4" s="2">
+        <f>COUNTA('1ST'!Q82:Q121)+COUNTA('2nd'!Q82:Q121)+COUNTA('3rd'!Q82:Q121)+COUNTA('4th'!Q82:Q121)+COUNTA('5th'!Q82:Q121)+COUNTA('6th'!Q82:Q121)+COUNTA('7th'!Q82:Q121)+COUNTA('8th'!Q82:Q121)+COUNTA('9th'!Q82:Q121)+COUNTA('10th'!Q82:Q121)+COUNTA('11th'!Q82:Q121)+COUNTA('12th'!Q82:Q121)+COUNTA('13th'!Q82:Q121)+COUNTA('14th'!Q82:Q121)+COUNTA('15th'!Q82:Q121)+COUNTA('16th'!Q82:Q121)+COUNTA('17th'!Q82:Q121)+COUNTA('18th'!Q82:Q121)+COUNTA('19th'!Q82:Q121)+COUNTA('20th'!Q82:Q121)+COUNTA('21st'!Q82:Q121)+COUNTA('22nd'!Q82:Q121)+COUNTA('23rd'!Q82:Q121)+COUNTA('24th'!Q82:Q121)+COUNTA('25th'!Q82:Q121)+COUNTA('26th'!Q82:Q121)+COUNTA('27th'!Q82:Q121)+COUNTA('28th'!Q82:Q121)+COUNTA('29th'!Q82:Q121)+COUNTA('30th'!Q82:Q121)+COUNTA('31st'!Q82:Q121)</f>
+        <v/>
+      </c>
+      <c r="R4" s="2">
+        <f>COUNTA('1ST'!R82:R121)+COUNTA('2nd'!R82:R121)+COUNTA('3rd'!R82:R121)+COUNTA('4th'!R82:R121)+COUNTA('5th'!R82:R121)+COUNTA('6th'!R82:R121)+COUNTA('7th'!R82:R121)+COUNTA('8th'!R82:R121)+COUNTA('9th'!R82:R121)+COUNTA('10th'!R82:R121)+COUNTA('11th'!R82:R121)+COUNTA('12th'!R82:R121)+COUNTA('13th'!R82:R121)+COUNTA('14th'!R82:R121)+COUNTA('15th'!R82:R121)+COUNTA('16th'!R82:R121)+COUNTA('17th'!R82:R121)+COUNTA('18th'!R82:R121)+COUNTA('19th'!R82:R121)+COUNTA('20th'!R82:R121)+COUNTA('21st'!R82:R121)+COUNTA('22nd'!R82:R121)+COUNTA('23rd'!R82:R121)+COUNTA('24th'!R82:R121)+COUNTA('25th'!R82:R121)+COUNTA('26th'!R82:R121)+COUNTA('27th'!R82:R121)+COUNTA('28th'!R82:R121)+COUNTA('29th'!R82:R121)+COUNTA('30th'!R82:R121)+COUNTA('31st'!R82:R121)</f>
+        <v/>
+      </c>
+      <c r="S4" s="2">
+        <f>COUNTA('1ST'!S82:S121)+COUNTA('2nd'!S82:S121)+COUNTA('3rd'!S82:S121)+COUNTA('4th'!S82:S121)+COUNTA('5th'!S82:S121)+COUNTA('6th'!S82:S121)+COUNTA('7th'!S82:S121)+COUNTA('8th'!S82:S121)+COUNTA('9th'!S82:S121)+COUNTA('10th'!S82:S121)+COUNTA('11th'!S82:S121)+COUNTA('12th'!S82:S121)+COUNTA('13th'!S82:S121)+COUNTA('14th'!S82:S121)+COUNTA('15th'!S82:S121)+COUNTA('16th'!S82:S121)+COUNTA('17th'!S82:S121)+COUNTA('18th'!S82:S121)+COUNTA('19th'!S82:S121)+COUNTA('20th'!S82:S121)+COUNTA('21st'!S82:S121)+COUNTA('22nd'!S82:S121)+COUNTA('23rd'!S82:S121)+COUNTA('24th'!S82:S121)+COUNTA('25th'!S82:S121)+COUNTA('26th'!S82:S121)+COUNTA('27th'!S82:S121)+COUNTA('28th'!S82:S121)+COUNTA('29th'!S82:S121)+COUNTA('30th'!S82:S121)+COUNTA('31st'!S82:S121)</f>
+        <v/>
+      </c>
+      <c r="T4" s="2">
+        <f>COUNTA('1ST'!T82:T121)+COUNTA('2nd'!T82:T121)+COUNTA('3rd'!T82:T121)+COUNTA('4th'!T82:T121)+COUNTA('5th'!T82:T121)+COUNTA('6th'!T82:T121)+COUNTA('7th'!T82:T121)+COUNTA('8th'!T82:T121)+COUNTA('9th'!T82:T121)+COUNTA('10th'!T82:T121)+COUNTA('11th'!T82:T121)+COUNTA('12th'!T82:T121)+COUNTA('13th'!T82:T121)+COUNTA('14th'!T82:T121)+COUNTA('15th'!T82:T121)+COUNTA('16th'!T82:T121)+COUNTA('17th'!T82:T121)+COUNTA('18th'!T82:T121)+COUNTA('19th'!T82:T121)+COUNTA('20th'!T82:T121)+COUNTA('21st'!T82:T121)+COUNTA('22nd'!T82:T121)+COUNTA('23rd'!T82:T121)+COUNTA('24th'!T82:T121)+COUNTA('25th'!T82:T121)+COUNTA('26th'!T82:T121)+COUNTA('27th'!T82:T121)+COUNTA('28th'!T82:T121)+COUNTA('29th'!T82:T121)+COUNTA('30th'!T82:T121)+COUNTA('31st'!T82:T121)</f>
+        <v/>
+      </c>
+      <c r="U4" s="2">
+        <f>COUNTA('1ST'!U82:U121)+COUNTA('2nd'!U82:U121)+COUNTA('3rd'!U82:U121)+COUNTA('4th'!U82:U121)+COUNTA('5th'!U82:U121)+COUNTA('6th'!U82:U121)+COUNTA('7th'!U82:U121)+COUNTA('8th'!U82:U121)+COUNTA('9th'!U82:U121)+COUNTA('10th'!U82:U121)+COUNTA('11th'!U82:U121)+COUNTA('12th'!U82:U121)+COUNTA('13th'!U82:U121)+COUNTA('14th'!U82:U121)+COUNTA('15th'!U82:U121)+COUNTA('16th'!U82:U121)+COUNTA('17th'!U82:U121)+COUNTA('18th'!U82:U121)+COUNTA('19th'!U82:U121)+COUNTA('20th'!U82:U121)+COUNTA('21st'!U82:U121)+COUNTA('22nd'!U82:U121)+COUNTA('23rd'!U82:U121)+COUNTA('24th'!U82:U121)+COUNTA('25th'!U82:U121)+COUNTA('26th'!U82:U121)+COUNTA('27th'!U82:U121)+COUNTA('28th'!U82:U121)+COUNTA('29th'!U82:U121)+COUNTA('30th'!U82:U121)+COUNTA('31st'!U82:U121)</f>
+        <v/>
+      </c>
       <c r="W4" s="4" t="n">
         <v>2</v>
       </c>
       <c r="AB4" s="4" t="n">
         <v>2</v>
       </c>
+      <c r="AG4" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="AL4" s="4" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Rinki Kumari</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>FC</t>
+        </is>
+      </c>
+      <c r="C5" s="2">
+        <f>COUNTA('1ST'!C122:C161)+COUNTA('2nd'!C122:C161)+COUNTA('3rd'!C122:C161)+COUNTA('4th'!C122:C161)+COUNTA('5th'!C122:C161)+COUNTA('6th'!C122:C161)+COUNTA('7th'!C122:C161)+COUNTA('8th'!C122:C161)+COUNTA('9th'!C122:C161)+COUNTA('10th'!C122:C161)+COUNTA('11th'!C122:C161)+COUNTA('12th'!C122:C161)+COUNTA('13th'!C122:C161)+COUNTA('14th'!C122:C161)+COUNTA('15th'!C122:C161)+COUNTA('16th'!C122:C161)+COUNTA('17th'!C122:C161)+COUNTA('18th'!C122:C161)+COUNTA('19th'!C122:C161)+COUNTA('20th'!C122:C161)+COUNTA('21st'!C122:C161)+COUNTA('22nd'!C122:C161)+COUNTA('23rd'!C122:C161)+COUNTA('24th'!C122:C161)+COUNTA('25th'!C122:C161)+COUNTA('26th'!C122:C161)+COUNTA('27th'!C122:C161)+COUNTA('28th'!C122:C161)+COUNTA('29th'!C122:C161)+COUNTA('30th'!C122:C161)+COUNTA('31st'!C122:C161)</f>
+        <v/>
+      </c>
+      <c r="D5" s="2">
+        <f>COUNTA('1ST'!D122:D161)+COUNTA('2nd'!D122:D161)+COUNTA('3rd'!D122:D161)+COUNTA('4th'!D122:D161)+COUNTA('5th'!D122:D161)+COUNTA('6th'!D122:D161)+COUNTA('7th'!D122:D161)+COUNTA('8th'!D122:D161)+COUNTA('9th'!D122:D161)+COUNTA('10th'!D122:D161)+COUNTA('11th'!D122:D161)+COUNTA('12th'!D122:D161)+COUNTA('13th'!D122:D161)+COUNTA('14th'!D122:D161)+COUNTA('15th'!D122:D161)+COUNTA('16th'!D122:D161)+COUNTA('17th'!D122:D161)+COUNTA('18th'!D122:D161)+COUNTA('19th'!D122:D161)+COUNTA('20th'!D122:D161)+COUNTA('21st'!D122:D161)+COUNTA('22nd'!D122:D161)+COUNTA('23rd'!D122:D161)+COUNTA('24th'!D122:D161)+COUNTA('25th'!D122:D161)+COUNTA('26th'!D122:D161)+COUNTA('27th'!D122:D161)+COUNTA('28th'!D122:D161)+COUNTA('29th'!D122:D161)+COUNTA('30th'!D122:D161)+COUNTA('31st'!D122:D161)</f>
+        <v/>
+      </c>
+      <c r="E5" s="2">
+        <f>COUNTA('1ST'!E122:E161)+COUNTA('2nd'!E122:E161)+COUNTA('3rd'!E122:E161)+COUNTA('4th'!E122:E161)+COUNTA('5th'!E122:E161)+COUNTA('6th'!E122:E161)+COUNTA('7th'!E122:E161)+COUNTA('8th'!E122:E161)+COUNTA('9th'!E122:E161)+COUNTA('10th'!E122:E161)+COUNTA('11th'!E122:E161)+COUNTA('12th'!E122:E161)+COUNTA('13th'!E122:E161)+COUNTA('14th'!E122:E161)+COUNTA('15th'!E122:E161)+COUNTA('16th'!E122:E161)+COUNTA('17th'!E122:E161)+COUNTA('18th'!E122:E161)+COUNTA('19th'!E122:E161)+COUNTA('20th'!E122:E161)+COUNTA('21st'!E122:E161)+COUNTA('22nd'!E122:E161)+COUNTA('23rd'!E122:E161)+COUNTA('24th'!E122:E161)+COUNTA('25th'!E122:E161)+COUNTA('26th'!E122:E161)+COUNTA('27th'!E122:E161)+COUNTA('28th'!E122:E161)+COUNTA('29th'!E122:E161)+COUNTA('30th'!E122:E161)+COUNTA('31st'!E122:E161)</f>
+        <v/>
+      </c>
+      <c r="F5" s="2">
+        <f>COUNTA('1ST'!F122:F161)+COUNTA('2nd'!F122:F161)+COUNTA('3rd'!F122:F161)+COUNTA('4th'!F122:F161)+COUNTA('5th'!F122:F161)+COUNTA('6th'!F122:F161)+COUNTA('7th'!F122:F161)+COUNTA('8th'!F122:F161)+COUNTA('9th'!F122:F161)+COUNTA('10th'!F122:F161)+COUNTA('11th'!F122:F161)+COUNTA('12th'!F122:F161)+COUNTA('13th'!F122:F161)+COUNTA('14th'!F122:F161)+COUNTA('15th'!F122:F161)+COUNTA('16th'!F122:F161)+COUNTA('17th'!F122:F161)+COUNTA('18th'!F122:F161)+COUNTA('19th'!F122:F161)+COUNTA('20th'!F122:F161)+COUNTA('21st'!F122:F161)+COUNTA('22nd'!F122:F161)+COUNTA('23rd'!F122:F161)+COUNTA('24th'!F122:F161)+COUNTA('25th'!F122:F161)+COUNTA('26th'!F122:F161)+COUNTA('27th'!F122:F161)+COUNTA('28th'!F122:F161)+COUNTA('29th'!F122:F161)+COUNTA('30th'!F122:F161)+COUNTA('31st'!F122:F161)</f>
+        <v/>
+      </c>
+      <c r="G5" s="2">
+        <f>COUNTA('1ST'!G122:G161)+COUNTA('2nd'!G122:G161)+COUNTA('3rd'!G122:G161)+COUNTA('4th'!G122:G161)+COUNTA('5th'!G122:G161)+COUNTA('6th'!G122:G161)+COUNTA('7th'!G122:G161)+COUNTA('8th'!G122:G161)+COUNTA('9th'!G122:G161)+COUNTA('10th'!G122:G161)+COUNTA('11th'!G122:G161)+COUNTA('12th'!G122:G161)+COUNTA('13th'!G122:G161)+COUNTA('14th'!G122:G161)+COUNTA('15th'!G122:G161)+COUNTA('16th'!G122:G161)+COUNTA('17th'!G122:G161)+COUNTA('18th'!G122:G161)+COUNTA('19th'!G122:G161)+COUNTA('20th'!G122:G161)+COUNTA('21st'!G122:G161)+COUNTA('22nd'!G122:G161)+COUNTA('23rd'!G122:G161)+COUNTA('24th'!G122:G161)+COUNTA('25th'!G122:G161)+COUNTA('26th'!G122:G161)+COUNTA('27th'!G122:G161)+COUNTA('28th'!G122:G161)+COUNTA('29th'!G122:G161)+COUNTA('30th'!G122:G161)+COUNTA('31st'!G122:G161)</f>
+        <v/>
+      </c>
+      <c r="H5" s="2">
+        <f>COUNTA('1ST'!H122:H161)+COUNTA('2nd'!H122:H161)+COUNTA('3rd'!H122:H161)+COUNTA('4th'!H122:H161)+COUNTA('5th'!H122:H161)+COUNTA('6th'!H122:H161)+COUNTA('7th'!H122:H161)+COUNTA('8th'!H122:H161)+COUNTA('9th'!H122:H161)+COUNTA('10th'!H122:H161)+COUNTA('11th'!H122:H161)+COUNTA('12th'!H122:H161)+COUNTA('13th'!H122:H161)+COUNTA('14th'!H122:H161)+COUNTA('15th'!H122:H161)+COUNTA('16th'!H122:H161)+COUNTA('17th'!H122:H161)+COUNTA('18th'!H122:H161)+COUNTA('19th'!H122:H161)+COUNTA('20th'!H122:H161)+COUNTA('21st'!H122:H161)+COUNTA('22nd'!H122:H161)+COUNTA('23rd'!H122:H161)+COUNTA('24th'!H122:H161)+COUNTA('25th'!H122:H161)+COUNTA('26th'!H122:H161)+COUNTA('27th'!H122:H161)+COUNTA('28th'!H122:H161)+COUNTA('29th'!H122:H161)+COUNTA('30th'!H122:H161)+COUNTA('31st'!H122:H161)</f>
+        <v/>
+      </c>
+      <c r="I5" s="2">
+        <f>COUNTA('1ST'!I122:I161)+COUNTA('2nd'!I122:I161)+COUNTA('3rd'!I122:I161)+COUNTA('4th'!I122:I161)+COUNTA('5th'!I122:I161)+COUNTA('6th'!I122:I161)+COUNTA('7th'!I122:I161)+COUNTA('8th'!I122:I161)+COUNTA('9th'!I122:I161)+COUNTA('10th'!I122:I161)+COUNTA('11th'!I122:I161)+COUNTA('12th'!I122:I161)+COUNTA('13th'!I122:I161)+COUNTA('14th'!I122:I161)+COUNTA('15th'!I122:I161)+COUNTA('16th'!I122:I161)+COUNTA('17th'!I122:I161)+COUNTA('18th'!I122:I161)+COUNTA('19th'!I122:I161)+COUNTA('20th'!I122:I161)+COUNTA('21st'!I122:I161)+COUNTA('22nd'!I122:I161)+COUNTA('23rd'!I122:I161)+COUNTA('24th'!I122:I161)+COUNTA('25th'!I122:I161)+COUNTA('26th'!I122:I161)+COUNTA('27th'!I122:I161)+COUNTA('28th'!I122:I161)+COUNTA('29th'!I122:I161)+COUNTA('30th'!I122:I161)+COUNTA('31st'!I122:I161)</f>
+        <v/>
+      </c>
+      <c r="J5" s="2">
+        <f>COUNTA('1ST'!J122:J161)+COUNTA('2nd'!J122:J161)+COUNTA('3rd'!J122:J161)+COUNTA('4th'!J122:J161)+COUNTA('5th'!J122:J161)+COUNTA('6th'!J122:J161)+COUNTA('7th'!J122:J161)+COUNTA('8th'!J122:J161)+COUNTA('9th'!J122:J161)+COUNTA('10th'!J122:J161)+COUNTA('11th'!J122:J161)+COUNTA('12th'!J122:J161)+COUNTA('13th'!J122:J161)+COUNTA('14th'!J122:J161)+COUNTA('15th'!J122:J161)+COUNTA('16th'!J122:J161)+COUNTA('17th'!J122:J161)+COUNTA('18th'!J122:J161)+COUNTA('19th'!J122:J161)+COUNTA('20th'!J122:J161)+COUNTA('21st'!J122:J161)+COUNTA('22nd'!J122:J161)+COUNTA('23rd'!J122:J161)+COUNTA('24th'!J122:J161)+COUNTA('25th'!J122:J161)+COUNTA('26th'!J122:J161)+COUNTA('27th'!J122:J161)+COUNTA('28th'!J122:J161)+COUNTA('29th'!J122:J161)+COUNTA('30th'!J122:J161)+COUNTA('31st'!J122:J161)</f>
+        <v/>
+      </c>
+      <c r="K5" s="2">
+        <f>COUNTA('1ST'!K122:K161)+COUNTA('2nd'!K122:K161)+COUNTA('3rd'!K122:K161)+COUNTA('4th'!K122:K161)+COUNTA('5th'!K122:K161)+COUNTA('6th'!K122:K161)+COUNTA('7th'!K122:K161)+COUNTA('8th'!K122:K161)+COUNTA('9th'!K122:K161)+COUNTA('10th'!K122:K161)+COUNTA('11th'!K122:K161)+COUNTA('12th'!K122:K161)+COUNTA('13th'!K122:K161)+COUNTA('14th'!K122:K161)+COUNTA('15th'!K122:K161)+COUNTA('16th'!K122:K161)+COUNTA('17th'!K122:K161)+COUNTA('18th'!K122:K161)+COUNTA('19th'!K122:K161)+COUNTA('20th'!K122:K161)+COUNTA('21st'!K122:K161)+COUNTA('22nd'!K122:K161)+COUNTA('23rd'!K122:K161)+COUNTA('24th'!K122:K161)+COUNTA('25th'!K122:K161)+COUNTA('26th'!K122:K161)+COUNTA('27th'!K122:K161)+COUNTA('28th'!K122:K161)+COUNTA('29th'!K122:K161)+COUNTA('30th'!K122:K161)+COUNTA('31st'!K122:K161)</f>
+        <v/>
+      </c>
+      <c r="L5" s="2">
+        <f>COUNTA('1ST'!L122:L161)+COUNTA('2nd'!L122:L161)+COUNTA('3rd'!L122:L161)+COUNTA('4th'!L122:L161)+COUNTA('5th'!L122:L161)+COUNTA('6th'!L122:L161)+COUNTA('7th'!L122:L161)+COUNTA('8th'!L122:L161)+COUNTA('9th'!L122:L161)+COUNTA('10th'!L122:L161)+COUNTA('11th'!L122:L161)+COUNTA('12th'!L122:L161)+COUNTA('13th'!L122:L161)+COUNTA('14th'!L122:L161)+COUNTA('15th'!L122:L161)+COUNTA('16th'!L122:L161)+COUNTA('17th'!L122:L161)+COUNTA('18th'!L122:L161)+COUNTA('19th'!L122:L161)+COUNTA('20th'!L122:L161)+COUNTA('21st'!L122:L161)+COUNTA('22nd'!L122:L161)+COUNTA('23rd'!L122:L161)+COUNTA('24th'!L122:L161)+COUNTA('25th'!L122:L161)+COUNTA('26th'!L122:L161)+COUNTA('27th'!L122:L161)+COUNTA('28th'!L122:L161)+COUNTA('29th'!L122:L161)+COUNTA('30th'!L122:L161)+COUNTA('31st'!L122:L161)</f>
+        <v/>
+      </c>
+      <c r="M5" s="2">
+        <f>COUNTA('1ST'!M122:M161)+COUNTA('2nd'!M122:M161)+COUNTA('3rd'!M122:M161)+COUNTA('4th'!M122:M161)+COUNTA('5th'!M122:M161)+COUNTA('6th'!M122:M161)+COUNTA('7th'!M122:M161)+COUNTA('8th'!M122:M161)+COUNTA('9th'!M122:M161)+COUNTA('10th'!M122:M161)+COUNTA('11th'!M122:M161)+COUNTA('12th'!M122:M161)+COUNTA('13th'!M122:M161)+COUNTA('14th'!M122:M161)+COUNTA('15th'!M122:M161)+COUNTA('16th'!M122:M161)+COUNTA('17th'!M122:M161)+COUNTA('18th'!M122:M161)+COUNTA('19th'!M122:M161)+COUNTA('20th'!M122:M161)+COUNTA('21st'!M122:M161)+COUNTA('22nd'!M122:M161)+COUNTA('23rd'!M122:M161)+COUNTA('24th'!M122:M161)+COUNTA('25th'!M122:M161)+COUNTA('26th'!M122:M161)+COUNTA('27th'!M122:M161)+COUNTA('28th'!M122:M161)+COUNTA('29th'!M122:M161)+COUNTA('30th'!M122:M161)+COUNTA('31st'!M122:M161)</f>
+        <v/>
+      </c>
+      <c r="N5" s="2">
+        <f>COUNTA('1ST'!N122:N161)+COUNTA('2nd'!N122:N161)+COUNTA('3rd'!N122:N161)+COUNTA('4th'!N122:N161)+COUNTA('5th'!N122:N161)+COUNTA('6th'!N122:N161)+COUNTA('7th'!N122:N161)+COUNTA('8th'!N122:N161)+COUNTA('9th'!N122:N161)+COUNTA('10th'!N122:N161)+COUNTA('11th'!N122:N161)+COUNTA('12th'!N122:N161)+COUNTA('13th'!N122:N161)+COUNTA('14th'!N122:N161)+COUNTA('15th'!N122:N161)+COUNTA('16th'!N122:N161)+COUNTA('17th'!N122:N161)+COUNTA('18th'!N122:N161)+COUNTA('19th'!N122:N161)+COUNTA('20th'!N122:N161)+COUNTA('21st'!N122:N161)+COUNTA('22nd'!N122:N161)+COUNTA('23rd'!N122:N161)+COUNTA('24th'!N122:N161)+COUNTA('25th'!N122:N161)+COUNTA('26th'!N122:N161)+COUNTA('27th'!N122:N161)+COUNTA('28th'!N122:N161)+COUNTA('29th'!N122:N161)+COUNTA('30th'!N122:N161)+COUNTA('31st'!N122:N161)</f>
+        <v/>
+      </c>
+      <c r="O5" s="2">
+        <f>COUNTA('1ST'!O122:O161)+COUNTA('2nd'!O122:O161)+COUNTA('3rd'!O122:O161)+COUNTA('4th'!O122:O161)+COUNTA('5th'!O122:O161)+COUNTA('6th'!O122:O161)+COUNTA('7th'!O122:O161)+COUNTA('8th'!O122:O161)+COUNTA('9th'!O122:O161)+COUNTA('10th'!O122:O161)+COUNTA('11th'!O122:O161)+COUNTA('12th'!O122:O161)+COUNTA('13th'!O122:O161)+COUNTA('14th'!O122:O161)+COUNTA('15th'!O122:O161)+COUNTA('16th'!O122:O161)+COUNTA('17th'!O122:O161)+COUNTA('18th'!O122:O161)+COUNTA('19th'!O122:O161)+COUNTA('20th'!O122:O161)+COUNTA('21st'!O122:O161)+COUNTA('22nd'!O122:O161)+COUNTA('23rd'!O122:O161)+COUNTA('24th'!O122:O161)+COUNTA('25th'!O122:O161)+COUNTA('26th'!O122:O161)+COUNTA('27th'!O122:O161)+COUNTA('28th'!O122:O161)+COUNTA('29th'!O122:O161)+COUNTA('30th'!O122:O161)+COUNTA('31st'!O122:O161)</f>
+        <v/>
+      </c>
+      <c r="P5" s="2">
+        <f>COUNTA('1ST'!P122:P161)+COUNTA('2nd'!P122:P161)+COUNTA('3rd'!P122:P161)+COUNTA('4th'!P122:P161)+COUNTA('5th'!P122:P161)+COUNTA('6th'!P122:P161)+COUNTA('7th'!P122:P161)+COUNTA('8th'!P122:P161)+COUNTA('9th'!P122:P161)+COUNTA('10th'!P122:P161)+COUNTA('11th'!P122:P161)+COUNTA('12th'!P122:P161)+COUNTA('13th'!P122:P161)+COUNTA('14th'!P122:P161)+COUNTA('15th'!P122:P161)+COUNTA('16th'!P122:P161)+COUNTA('17th'!P122:P161)+COUNTA('18th'!P122:P161)+COUNTA('19th'!P122:P161)+COUNTA('20th'!P122:P161)+COUNTA('21st'!P122:P161)+COUNTA('22nd'!P122:P161)+COUNTA('23rd'!P122:P161)+COUNTA('24th'!P122:P161)+COUNTA('25th'!P122:P161)+COUNTA('26th'!P122:P161)+COUNTA('27th'!P122:P161)+COUNTA('28th'!P122:P161)+COUNTA('29th'!P122:P161)+COUNTA('30th'!P122:P161)+COUNTA('31st'!P122:P161)</f>
+        <v/>
+      </c>
+      <c r="Q5" s="2">
+        <f>COUNTA('1ST'!Q122:Q161)+COUNTA('2nd'!Q122:Q161)+COUNTA('3rd'!Q122:Q161)+COUNTA('4th'!Q122:Q161)+COUNTA('5th'!Q122:Q161)+COUNTA('6th'!Q122:Q161)+COUNTA('7th'!Q122:Q161)+COUNTA('8th'!Q122:Q161)+COUNTA('9th'!Q122:Q161)+COUNTA('10th'!Q122:Q161)+COUNTA('11th'!Q122:Q161)+COUNTA('12th'!Q122:Q161)+COUNTA('13th'!Q122:Q161)+COUNTA('14th'!Q122:Q161)+COUNTA('15th'!Q122:Q161)+COUNTA('16th'!Q122:Q161)+COUNTA('17th'!Q122:Q161)+COUNTA('18th'!Q122:Q161)+COUNTA('19th'!Q122:Q161)+COUNTA('20th'!Q122:Q161)+COUNTA('21st'!Q122:Q161)+COUNTA('22nd'!Q122:Q161)+COUNTA('23rd'!Q122:Q161)+COUNTA('24th'!Q122:Q161)+COUNTA('25th'!Q122:Q161)+COUNTA('26th'!Q122:Q161)+COUNTA('27th'!Q122:Q161)+COUNTA('28th'!Q122:Q161)+COUNTA('29th'!Q122:Q161)+COUNTA('30th'!Q122:Q161)+COUNTA('31st'!Q122:Q161)</f>
+        <v/>
+      </c>
+      <c r="R5" s="2">
+        <f>COUNTA('1ST'!R122:R161)+COUNTA('2nd'!R122:R161)+COUNTA('3rd'!R122:R161)+COUNTA('4th'!R122:R161)+COUNTA('5th'!R122:R161)+COUNTA('6th'!R122:R161)+COUNTA('7th'!R122:R161)+COUNTA('8th'!R122:R161)+COUNTA('9th'!R122:R161)+COUNTA('10th'!R122:R161)+COUNTA('11th'!R122:R161)+COUNTA('12th'!R122:R161)+COUNTA('13th'!R122:R161)+COUNTA('14th'!R122:R161)+COUNTA('15th'!R122:R161)+COUNTA('16th'!R122:R161)+COUNTA('17th'!R122:R161)+COUNTA('18th'!R122:R161)+COUNTA('19th'!R122:R161)+COUNTA('20th'!R122:R161)+COUNTA('21st'!R122:R161)+COUNTA('22nd'!R122:R161)+COUNTA('23rd'!R122:R161)+COUNTA('24th'!R122:R161)+COUNTA('25th'!R122:R161)+COUNTA('26th'!R122:R161)+COUNTA('27th'!R122:R161)+COUNTA('28th'!R122:R161)+COUNTA('29th'!R122:R161)+COUNTA('30th'!R122:R161)+COUNTA('31st'!R122:R161)</f>
+        <v/>
+      </c>
+      <c r="S5" s="2">
+        <f>COUNTA('1ST'!S122:S161)+COUNTA('2nd'!S122:S161)+COUNTA('3rd'!S122:S161)+COUNTA('4th'!S122:S161)+COUNTA('5th'!S122:S161)+COUNTA('6th'!S122:S161)+COUNTA('7th'!S122:S161)+COUNTA('8th'!S122:S161)+COUNTA('9th'!S122:S161)+COUNTA('10th'!S122:S161)+COUNTA('11th'!S122:S161)+COUNTA('12th'!S122:S161)+COUNTA('13th'!S122:S161)+COUNTA('14th'!S122:S161)+COUNTA('15th'!S122:S161)+COUNTA('16th'!S122:S161)+COUNTA('17th'!S122:S161)+COUNTA('18th'!S122:S161)+COUNTA('19th'!S122:S161)+COUNTA('20th'!S122:S161)+COUNTA('21st'!S122:S161)+COUNTA('22nd'!S122:S161)+COUNTA('23rd'!S122:S161)+COUNTA('24th'!S122:S161)+COUNTA('25th'!S122:S161)+COUNTA('26th'!S122:S161)+COUNTA('27th'!S122:S161)+COUNTA('28th'!S122:S161)+COUNTA('29th'!S122:S161)+COUNTA('30th'!S122:S161)+COUNTA('31st'!S122:S161)</f>
+        <v/>
+      </c>
+      <c r="T5" s="2">
+        <f>COUNTA('1ST'!T122:T161)+COUNTA('2nd'!T122:T161)+COUNTA('3rd'!T122:T161)+COUNTA('4th'!T122:T161)+COUNTA('5th'!T122:T161)+COUNTA('6th'!T122:T161)+COUNTA('7th'!T122:T161)+COUNTA('8th'!T122:T161)+COUNTA('9th'!T122:T161)+COUNTA('10th'!T122:T161)+COUNTA('11th'!T122:T161)+COUNTA('12th'!T122:T161)+COUNTA('13th'!T122:T161)+COUNTA('14th'!T122:T161)+COUNTA('15th'!T122:T161)+COUNTA('16th'!T122:T161)+COUNTA('17th'!T122:T161)+COUNTA('18th'!T122:T161)+COUNTA('19th'!T122:T161)+COUNTA('20th'!T122:T161)+COUNTA('21st'!T122:T161)+COUNTA('22nd'!T122:T161)+COUNTA('23rd'!T122:T161)+COUNTA('24th'!T122:T161)+COUNTA('25th'!T122:T161)+COUNTA('26th'!T122:T161)+COUNTA('27th'!T122:T161)+COUNTA('28th'!T122:T161)+COUNTA('29th'!T122:T161)+COUNTA('30th'!T122:T161)+COUNTA('31st'!T122:T161)</f>
+        <v/>
+      </c>
+      <c r="U5" s="2">
+        <f>COUNTA('1ST'!U122:U161)+COUNTA('2nd'!U122:U161)+COUNTA('3rd'!U122:U161)+COUNTA('4th'!U122:U161)+COUNTA('5th'!U122:U161)+COUNTA('6th'!U122:U161)+COUNTA('7th'!U122:U161)+COUNTA('8th'!U122:U161)+COUNTA('9th'!U122:U161)+COUNTA('10th'!U122:U161)+COUNTA('11th'!U122:U161)+COUNTA('12th'!U122:U161)+COUNTA('13th'!U122:U161)+COUNTA('14th'!U122:U161)+COUNTA('15th'!U122:U161)+COUNTA('16th'!U122:U161)+COUNTA('17th'!U122:U161)+COUNTA('18th'!U122:U161)+COUNTA('19th'!U122:U161)+COUNTA('20th'!U122:U161)+COUNTA('21st'!U122:U161)+COUNTA('22nd'!U122:U161)+COUNTA('23rd'!U122:U161)+COUNTA('24th'!U122:U161)+COUNTA('25th'!U122:U161)+COUNTA('26th'!U122:U161)+COUNTA('27th'!U122:U161)+COUNTA('28th'!U122:U161)+COUNTA('29th'!U122:U161)+COUNTA('30th'!U122:U161)+COUNTA('31st'!U122:U161)</f>
+        <v/>
+      </c>
       <c r="W5" s="4" t="n">
         <v>3</v>
       </c>
       <c r="AB5" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="AG5" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="AL5" s="4" t="n">
         <v>3</v>
       </c>
     </row>
@@ -3195,6 +3755,12 @@
       <c r="AB6" s="4" t="n">
         <v>4</v>
       </c>
+      <c r="AG6" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="AL6" s="4" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="7">
       <c r="W7" s="4" t="n">
@@ -3203,6 +3769,12 @@
       <c r="AB7" s="4" t="n">
         <v>5</v>
       </c>
+      <c r="AG7" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="AL7" s="4" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="8">
       <c r="W8" s="4" t="n">
@@ -3211,6 +3783,12 @@
       <c r="AB8" s="4" t="n">
         <v>6</v>
       </c>
+      <c r="AG8" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="AL8" s="4" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="9">
       <c r="W9" s="4" t="n">
@@ -3219,6 +3797,12 @@
       <c r="AB9" s="4" t="n">
         <v>7</v>
       </c>
+      <c r="AG9" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="AL9" s="4" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="10">
       <c r="W10" s="4" t="n">
@@ -3227,6 +3811,12 @@
       <c r="AB10" s="4" t="n">
         <v>8</v>
       </c>
+      <c r="AG10" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="AL10" s="4" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="11">
       <c r="W11" s="4" t="n">
@@ -3235,6 +3825,12 @@
       <c r="AB11" s="4" t="n">
         <v>9</v>
       </c>
+      <c r="AG11" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="AL11" s="4" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="12">
       <c r="W12" s="4" t="n">
@@ -3243,6 +3839,12 @@
       <c r="AB12" s="4" t="n">
         <v>10</v>
       </c>
+      <c r="AG12" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="AL12" s="4" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="13">
       <c r="W13" s="4" t="n">
@@ -3251,6 +3853,12 @@
       <c r="AB13" s="4" t="n">
         <v>11</v>
       </c>
+      <c r="AG13" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="AL13" s="4" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="14">
       <c r="W14" s="4" t="n">
@@ -3259,6 +3867,12 @@
       <c r="AB14" s="4" t="n">
         <v>12</v>
       </c>
+      <c r="AG14" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="AL14" s="4" t="n">
+        <v>12</v>
+      </c>
     </row>
     <row r="15">
       <c r="W15" s="4" t="n">
@@ -3267,6 +3881,12 @@
       <c r="AB15" s="4" t="n">
         <v>13</v>
       </c>
+      <c r="AG15" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="AL15" s="4" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="16">
       <c r="W16" s="4" t="n">
@@ -3275,6 +3895,12 @@
       <c r="AB16" s="4" t="n">
         <v>14</v>
       </c>
+      <c r="AG16" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="AL16" s="4" t="n">
+        <v>14</v>
+      </c>
     </row>
     <row r="17">
       <c r="W17" s="4" t="n">
@@ -3283,6 +3909,12 @@
       <c r="AB17" s="4" t="n">
         <v>15</v>
       </c>
+      <c r="AG17" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="AL17" s="4" t="n">
+        <v>15</v>
+      </c>
     </row>
     <row r="18">
       <c r="W18" s="4" t="n">
@@ -3291,6 +3923,12 @@
       <c r="AB18" s="4" t="n">
         <v>16</v>
       </c>
+      <c r="AG18" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="AL18" s="4" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="19">
       <c r="W19" s="4" t="n">
@@ -3299,6 +3937,12 @@
       <c r="AB19" s="4" t="n">
         <v>17</v>
       </c>
+      <c r="AG19" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="AL19" s="4" t="n">
+        <v>17</v>
+      </c>
     </row>
     <row r="20">
       <c r="W20" s="4" t="n">
@@ -3307,6 +3951,12 @@
       <c r="AB20" s="4" t="n">
         <v>18</v>
       </c>
+      <c r="AG20" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="AL20" s="4" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="21">
       <c r="W21" s="4" t="n">
@@ -3315,6 +3965,12 @@
       <c r="AB21" s="4" t="n">
         <v>19</v>
       </c>
+      <c r="AG21" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="AL21" s="4" t="n">
+        <v>19</v>
+      </c>
     </row>
     <row r="22">
       <c r="W22" s="4" t="n">
@@ -3323,6 +3979,12 @@
       <c r="AB22" s="4" t="n">
         <v>20</v>
       </c>
+      <c r="AG22" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="AL22" s="4" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="23">
       <c r="W23" s="4" t="n">
@@ -3331,6 +3993,12 @@
       <c r="AB23" s="4" t="n">
         <v>21</v>
       </c>
+      <c r="AG23" s="4" t="n">
+        <v>21</v>
+      </c>
+      <c r="AL23" s="4" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="24">
       <c r="W24" s="4" t="n">
@@ -3339,6 +4007,12 @@
       <c r="AB24" s="4" t="n">
         <v>22</v>
       </c>
+      <c r="AG24" s="4" t="n">
+        <v>22</v>
+      </c>
+      <c r="AL24" s="4" t="n">
+        <v>22</v>
+      </c>
     </row>
     <row r="25">
       <c r="W25" s="4" t="n">
@@ -3347,6 +4021,12 @@
       <c r="AB25" s="4" t="n">
         <v>23</v>
       </c>
+      <c r="AG25" s="4" t="n">
+        <v>23</v>
+      </c>
+      <c r="AL25" s="4" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="26">
       <c r="W26" s="4" t="n">
@@ -3355,6 +4035,12 @@
       <c r="AB26" s="4" t="n">
         <v>24</v>
       </c>
+      <c r="AG26" s="4" t="n">
+        <v>24</v>
+      </c>
+      <c r="AL26" s="4" t="n">
+        <v>24</v>
+      </c>
     </row>
     <row r="27">
       <c r="W27" s="4" t="n">
@@ -3363,6 +4049,12 @@
       <c r="AB27" s="4" t="n">
         <v>25</v>
       </c>
+      <c r="AG27" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="AL27" s="4" t="n">
+        <v>25</v>
+      </c>
     </row>
     <row r="28">
       <c r="W28" s="4" t="n">
@@ -3371,6 +4063,12 @@
       <c r="AB28" s="4" t="n">
         <v>26</v>
       </c>
+      <c r="AG28" s="4" t="n">
+        <v>26</v>
+      </c>
+      <c r="AL28" s="4" t="n">
+        <v>26</v>
+      </c>
     </row>
     <row r="29">
       <c r="W29" s="4" t="n">
@@ -3379,6 +4077,12 @@
       <c r="AB29" s="4" t="n">
         <v>27</v>
       </c>
+      <c r="AG29" s="4" t="n">
+        <v>27</v>
+      </c>
+      <c r="AL29" s="4" t="n">
+        <v>27</v>
+      </c>
     </row>
     <row r="30">
       <c r="W30" s="4" t="n">
@@ -3387,6 +4091,12 @@
       <c r="AB30" s="4" t="n">
         <v>28</v>
       </c>
+      <c r="AG30" s="4" t="n">
+        <v>28</v>
+      </c>
+      <c r="AL30" s="4" t="n">
+        <v>28</v>
+      </c>
     </row>
     <row r="31">
       <c r="W31" s="4" t="n">
@@ -3395,6 +4105,12 @@
       <c r="AB31" s="4" t="n">
         <v>29</v>
       </c>
+      <c r="AG31" s="4" t="n">
+        <v>29</v>
+      </c>
+      <c r="AL31" s="4" t="n">
+        <v>29</v>
+      </c>
     </row>
     <row r="32">
       <c r="W32" s="4" t="n">
@@ -3403,6 +4119,12 @@
       <c r="AB32" s="4" t="n">
         <v>30</v>
       </c>
+      <c r="AG32" s="4" t="n">
+        <v>30</v>
+      </c>
+      <c r="AL32" s="4" t="n">
+        <v>30</v>
+      </c>
     </row>
     <row r="33">
       <c r="W33" s="4" t="n">
@@ -3411,11 +4133,19 @@
       <c r="AB33" s="4" t="n">
         <v>31</v>
       </c>
+      <c r="AG33" s="4" t="n">
+        <v>31</v>
+      </c>
+      <c r="AL33" s="4" t="n">
+        <v>31</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="4">
     <mergeCell ref="AB1:AE1"/>
     <mergeCell ref="W1:Z1"/>
+    <mergeCell ref="AL1:AO1"/>
+    <mergeCell ref="AG1:AJ1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
@@ -3428,7 +4158,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U42"/>
+  <dimension ref="A1:U122"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -3564,24 +4294,48 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Rajiv Kumar</t>
+          <t>Bablu Kumar</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Field Officer</t>
+          <t>FC</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
+          <t>Monu Kumar</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>FC</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="inlineStr">
+        <is>
+          <t>Rajiv Kumar</t>
+        </is>
+      </c>
+      <c r="B82" s="2" t="inlineStr">
+        <is>
+          <t>FC</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="2" t="inlineStr">
+        <is>
           <t>Rinki Kumari</t>
         </is>
       </c>
-      <c r="B42" s="2" t="inlineStr">
-        <is>
-          <t>Field Officer</t>
+      <c r="B122" s="2" t="inlineStr">
+        <is>
+          <t>FC</t>
         </is>
       </c>
     </row>
@@ -3597,7 +4351,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U42"/>
+  <dimension ref="A1:U122"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -3733,24 +4487,48 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Rajiv Kumar</t>
+          <t>Bablu Kumar</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Field Officer</t>
+          <t>FC</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
+          <t>Monu Kumar</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>FC</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="inlineStr">
+        <is>
+          <t>Rajiv Kumar</t>
+        </is>
+      </c>
+      <c r="B82" s="2" t="inlineStr">
+        <is>
+          <t>FC</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="2" t="inlineStr">
+        <is>
           <t>Rinki Kumari</t>
         </is>
       </c>
-      <c r="B42" s="2" t="inlineStr">
-        <is>
-          <t>Field Officer</t>
+      <c r="B122" s="2" t="inlineStr">
+        <is>
+          <t>FC</t>
         </is>
       </c>
     </row>
@@ -3766,7 +4544,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U42"/>
+  <dimension ref="A1:U122"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -3902,24 +4680,48 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Rajiv Kumar</t>
+          <t>Bablu Kumar</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Field Officer</t>
+          <t>FC</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
+          <t>Monu Kumar</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>FC</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="inlineStr">
+        <is>
+          <t>Rajiv Kumar</t>
+        </is>
+      </c>
+      <c r="B82" s="2" t="inlineStr">
+        <is>
+          <t>FC</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="2" t="inlineStr">
+        <is>
           <t>Rinki Kumari</t>
         </is>
       </c>
-      <c r="B42" s="2" t="inlineStr">
-        <is>
-          <t>Field Officer</t>
+      <c r="B122" s="2" t="inlineStr">
+        <is>
+          <t>FC</t>
         </is>
       </c>
     </row>
@@ -3935,7 +4737,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U42"/>
+  <dimension ref="A1:U122"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -4071,24 +4873,48 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Rajiv Kumar</t>
+          <t>Bablu Kumar</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Field Officer</t>
+          <t>FC</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
+          <t>Monu Kumar</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>FC</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="inlineStr">
+        <is>
+          <t>Rajiv Kumar</t>
+        </is>
+      </c>
+      <c r="B82" s="2" t="inlineStr">
+        <is>
+          <t>FC</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="2" t="inlineStr">
+        <is>
           <t>Rinki Kumari</t>
         </is>
       </c>
-      <c r="B42" s="2" t="inlineStr">
-        <is>
-          <t>Field Officer</t>
+      <c r="B122" s="2" t="inlineStr">
+        <is>
+          <t>FC</t>
         </is>
       </c>
     </row>
@@ -4104,7 +4930,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U42"/>
+  <dimension ref="A1:U122"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -4240,24 +5066,48 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Rajiv Kumar</t>
+          <t>Bablu Kumar</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Field Officer</t>
+          <t>FC</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
+          <t>Monu Kumar</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>FC</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="inlineStr">
+        <is>
+          <t>Rajiv Kumar</t>
+        </is>
+      </c>
+      <c r="B82" s="2" t="inlineStr">
+        <is>
+          <t>FC</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="2" t="inlineStr">
+        <is>
           <t>Rinki Kumari</t>
         </is>
       </c>
-      <c r="B42" s="2" t="inlineStr">
-        <is>
-          <t>Field Officer</t>
+      <c r="B122" s="2" t="inlineStr">
+        <is>
+          <t>FC</t>
         </is>
       </c>
     </row>
@@ -4273,7 +5123,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U42"/>
+  <dimension ref="A1:U122"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -4409,24 +5259,48 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Rajiv Kumar</t>
+          <t>Bablu Kumar</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Field Officer</t>
+          <t>FC</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
+          <t>Monu Kumar</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>FC</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="inlineStr">
+        <is>
+          <t>Rajiv Kumar</t>
+        </is>
+      </c>
+      <c r="B82" s="2" t="inlineStr">
+        <is>
+          <t>FC</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="2" t="inlineStr">
+        <is>
           <t>Rinki Kumari</t>
         </is>
       </c>
-      <c r="B42" s="2" t="inlineStr">
-        <is>
-          <t>Field Officer</t>
+      <c r="B122" s="2" t="inlineStr">
+        <is>
+          <t>FC</t>
         </is>
       </c>
     </row>
@@ -4442,7 +5316,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U42"/>
+  <dimension ref="A1:U122"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -4578,24 +5452,48 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Rajiv Kumar</t>
+          <t>Bablu Kumar</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Field Officer</t>
+          <t>FC</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
+          <t>Monu Kumar</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>FC</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="inlineStr">
+        <is>
+          <t>Rajiv Kumar</t>
+        </is>
+      </c>
+      <c r="B82" s="2" t="inlineStr">
+        <is>
+          <t>FC</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="2" t="inlineStr">
+        <is>
           <t>Rinki Kumari</t>
         </is>
       </c>
-      <c r="B42" s="2" t="inlineStr">
-        <is>
-          <t>Field Officer</t>
+      <c r="B122" s="2" t="inlineStr">
+        <is>
+          <t>FC</t>
         </is>
       </c>
     </row>
@@ -4611,7 +5509,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U42"/>
+  <dimension ref="A1:U122"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -4747,24 +5645,48 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Rajiv Kumar</t>
+          <t>Bablu Kumar</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Field Officer</t>
+          <t>FC</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
+          <t>Monu Kumar</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>FC</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="inlineStr">
+        <is>
+          <t>Rajiv Kumar</t>
+        </is>
+      </c>
+      <c r="B82" s="2" t="inlineStr">
+        <is>
+          <t>FC</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="2" t="inlineStr">
+        <is>
           <t>Rinki Kumari</t>
         </is>
       </c>
-      <c r="B42" s="2" t="inlineStr">
-        <is>
-          <t>Field Officer</t>
+      <c r="B122" s="2" t="inlineStr">
+        <is>
+          <t>FC</t>
         </is>
       </c>
     </row>
@@ -4780,7 +5702,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U42"/>
+  <dimension ref="A1:U122"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -4916,24 +5838,48 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Rajiv Kumar</t>
+          <t>Bablu Kumar</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Field Officer</t>
+          <t>FC</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
+          <t>Monu Kumar</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>FC</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="inlineStr">
+        <is>
+          <t>Rajiv Kumar</t>
+        </is>
+      </c>
+      <c r="B82" s="2" t="inlineStr">
+        <is>
+          <t>FC</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="2" t="inlineStr">
+        <is>
           <t>Rinki Kumari</t>
         </is>
       </c>
-      <c r="B42" s="2" t="inlineStr">
-        <is>
-          <t>Field Officer</t>
+      <c r="B122" s="2" t="inlineStr">
+        <is>
+          <t>FC</t>
         </is>
       </c>
     </row>
@@ -4949,7 +5895,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U42"/>
+  <dimension ref="A1:U122"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -5085,24 +6031,48 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Rajiv Kumar</t>
+          <t>Bablu Kumar</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Field Officer</t>
+          <t>FC</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
+          <t>Monu Kumar</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>FC</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="inlineStr">
+        <is>
+          <t>Rajiv Kumar</t>
+        </is>
+      </c>
+      <c r="B82" s="2" t="inlineStr">
+        <is>
+          <t>FC</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="2" t="inlineStr">
+        <is>
           <t>Rinki Kumari</t>
         </is>
       </c>
-      <c r="B42" s="2" t="inlineStr">
-        <is>
-          <t>Field Officer</t>
+      <c r="B122" s="2" t="inlineStr">
+        <is>
+          <t>FC</t>
         </is>
       </c>
     </row>
@@ -5118,7 +6088,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U42"/>
+  <dimension ref="A1:U122"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -5254,24 +6224,48 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Rajiv Kumar</t>
+          <t>Bablu Kumar</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Field Officer</t>
+          <t>FC</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
+          <t>Monu Kumar</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>FC</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="inlineStr">
+        <is>
+          <t>Rajiv Kumar</t>
+        </is>
+      </c>
+      <c r="B82" s="2" t="inlineStr">
+        <is>
+          <t>FC</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="2" t="inlineStr">
+        <is>
           <t>Rinki Kumari</t>
         </is>
       </c>
-      <c r="B42" s="2" t="inlineStr">
-        <is>
-          <t>Field Officer</t>
+      <c r="B122" s="2" t="inlineStr">
+        <is>
+          <t>FC</t>
         </is>
       </c>
     </row>
@@ -5287,7 +6281,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U42"/>
+  <dimension ref="A1:U122"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -5423,24 +6417,48 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Rajiv Kumar</t>
+          <t>Bablu Kumar</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Field Officer</t>
+          <t>FC</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
+          <t>Monu Kumar</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>FC</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="inlineStr">
+        <is>
+          <t>Rajiv Kumar</t>
+        </is>
+      </c>
+      <c r="B82" s="2" t="inlineStr">
+        <is>
+          <t>FC</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="2" t="inlineStr">
+        <is>
           <t>Rinki Kumari</t>
         </is>
       </c>
-      <c r="B42" s="2" t="inlineStr">
-        <is>
-          <t>Field Officer</t>
+      <c r="B122" s="2" t="inlineStr">
+        <is>
+          <t>FC</t>
         </is>
       </c>
     </row>
@@ -5456,7 +6474,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U42"/>
+  <dimension ref="A1:U122"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -5592,24 +6610,48 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Rajiv Kumar</t>
+          <t>Bablu Kumar</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Field Officer</t>
+          <t>FC</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
+          <t>Monu Kumar</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>FC</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="inlineStr">
+        <is>
+          <t>Rajiv Kumar</t>
+        </is>
+      </c>
+      <c r="B82" s="2" t="inlineStr">
+        <is>
+          <t>FC</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="2" t="inlineStr">
+        <is>
           <t>Rinki Kumari</t>
         </is>
       </c>
-      <c r="B42" s="2" t="inlineStr">
-        <is>
-          <t>Field Officer</t>
+      <c r="B122" s="2" t="inlineStr">
+        <is>
+          <t>FC</t>
         </is>
       </c>
     </row>
@@ -5625,7 +6667,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U42"/>
+  <dimension ref="A1:U122"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -5761,24 +6803,48 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Rajiv Kumar</t>
+          <t>Bablu Kumar</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Field Officer</t>
+          <t>FC</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
+          <t>Monu Kumar</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>FC</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="inlineStr">
+        <is>
+          <t>Rajiv Kumar</t>
+        </is>
+      </c>
+      <c r="B82" s="2" t="inlineStr">
+        <is>
+          <t>FC</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="2" t="inlineStr">
+        <is>
           <t>Rinki Kumari</t>
         </is>
       </c>
-      <c r="B42" s="2" t="inlineStr">
-        <is>
-          <t>Field Officer</t>
+      <c r="B122" s="2" t="inlineStr">
+        <is>
+          <t>FC</t>
         </is>
       </c>
     </row>
@@ -5794,7 +6860,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U42"/>
+  <dimension ref="A1:U122"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -5930,24 +6996,48 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Rajiv Kumar</t>
+          <t>Bablu Kumar</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Field Officer</t>
+          <t>FC</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
+          <t>Monu Kumar</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>FC</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="inlineStr">
+        <is>
+          <t>Rajiv Kumar</t>
+        </is>
+      </c>
+      <c r="B82" s="2" t="inlineStr">
+        <is>
+          <t>FC</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="2" t="inlineStr">
+        <is>
           <t>Rinki Kumari</t>
         </is>
       </c>
-      <c r="B42" s="2" t="inlineStr">
-        <is>
-          <t>Field Officer</t>
+      <c r="B122" s="2" t="inlineStr">
+        <is>
+          <t>FC</t>
         </is>
       </c>
     </row>
@@ -5963,7 +7053,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U42"/>
+  <dimension ref="A1:U122"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -6099,24 +7189,48 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Rajiv Kumar</t>
+          <t>Bablu Kumar</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Field Officer</t>
+          <t>FC</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
+          <t>Monu Kumar</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>FC</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="inlineStr">
+        <is>
+          <t>Rajiv Kumar</t>
+        </is>
+      </c>
+      <c r="B82" s="2" t="inlineStr">
+        <is>
+          <t>FC</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="2" t="inlineStr">
+        <is>
           <t>Rinki Kumari</t>
         </is>
       </c>
-      <c r="B42" s="2" t="inlineStr">
-        <is>
-          <t>Field Officer</t>
+      <c r="B122" s="2" t="inlineStr">
+        <is>
+          <t>FC</t>
         </is>
       </c>
     </row>
@@ -6132,7 +7246,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U42"/>
+  <dimension ref="A1:U122"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -6268,24 +7382,48 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Rajiv Kumar</t>
+          <t>Bablu Kumar</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Field Officer</t>
+          <t>FC</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
+          <t>Monu Kumar</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>FC</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="inlineStr">
+        <is>
+          <t>Rajiv Kumar</t>
+        </is>
+      </c>
+      <c r="B82" s="2" t="inlineStr">
+        <is>
+          <t>FC</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="2" t="inlineStr">
+        <is>
           <t>Rinki Kumari</t>
         </is>
       </c>
-      <c r="B42" s="2" t="inlineStr">
-        <is>
-          <t>Field Officer</t>
+      <c r="B122" s="2" t="inlineStr">
+        <is>
+          <t>FC</t>
         </is>
       </c>
     </row>
@@ -6301,7 +7439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U42"/>
+  <dimension ref="A1:U122"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -6437,24 +7575,48 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Rajiv Kumar</t>
+          <t>Bablu Kumar</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Field Officer</t>
+          <t>FC</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
+          <t>Monu Kumar</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>FC</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="inlineStr">
+        <is>
+          <t>Rajiv Kumar</t>
+        </is>
+      </c>
+      <c r="B82" s="2" t="inlineStr">
+        <is>
+          <t>FC</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="2" t="inlineStr">
+        <is>
           <t>Rinki Kumari</t>
         </is>
       </c>
-      <c r="B42" s="2" t="inlineStr">
-        <is>
-          <t>Field Officer</t>
+      <c r="B122" s="2" t="inlineStr">
+        <is>
+          <t>FC</t>
         </is>
       </c>
     </row>
@@ -6470,7 +7632,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U42"/>
+  <dimension ref="A1:U122"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -6606,24 +7768,48 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Rajiv Kumar</t>
+          <t>Bablu Kumar</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Field Officer</t>
+          <t>FC</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
+          <t>Monu Kumar</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>FC</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="inlineStr">
+        <is>
+          <t>Rajiv Kumar</t>
+        </is>
+      </c>
+      <c r="B82" s="2" t="inlineStr">
+        <is>
+          <t>FC</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="2" t="inlineStr">
+        <is>
           <t>Rinki Kumari</t>
         </is>
       </c>
-      <c r="B42" s="2" t="inlineStr">
-        <is>
-          <t>Field Officer</t>
+      <c r="B122" s="2" t="inlineStr">
+        <is>
+          <t>FC</t>
         </is>
       </c>
     </row>
@@ -6639,7 +7825,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U42"/>
+  <dimension ref="A1:U122"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -6775,24 +7961,48 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Rajiv Kumar</t>
+          <t>Bablu Kumar</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Field Officer</t>
+          <t>FC</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
+          <t>Monu Kumar</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>FC</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="inlineStr">
+        <is>
+          <t>Rajiv Kumar</t>
+        </is>
+      </c>
+      <c r="B82" s="2" t="inlineStr">
+        <is>
+          <t>FC</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="2" t="inlineStr">
+        <is>
           <t>Rinki Kumari</t>
         </is>
       </c>
-      <c r="B42" s="2" t="inlineStr">
-        <is>
-          <t>Field Officer</t>
+      <c r="B122" s="2" t="inlineStr">
+        <is>
+          <t>FC</t>
         </is>
       </c>
     </row>
@@ -6808,7 +8018,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U42"/>
+  <dimension ref="A1:U122"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -6944,24 +8154,48 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Rajiv Kumar</t>
+          <t>Bablu Kumar</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Field Officer</t>
+          <t>FC</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
+          <t>Monu Kumar</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>FC</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="inlineStr">
+        <is>
+          <t>Rajiv Kumar</t>
+        </is>
+      </c>
+      <c r="B82" s="2" t="inlineStr">
+        <is>
+          <t>FC</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="2" t="inlineStr">
+        <is>
           <t>Rinki Kumari</t>
         </is>
       </c>
-      <c r="B42" s="2" t="inlineStr">
-        <is>
-          <t>Field Officer</t>
+      <c r="B122" s="2" t="inlineStr">
+        <is>
+          <t>FC</t>
         </is>
       </c>
     </row>

</xml_diff>